<commit_message>
Correct model names and update Camp photos and floorplans
</commit_message>
<xml_diff>
--- a/data/sources/OFFERED MODELS.xlsx
+++ b/data/sources/OFFERED MODELS.xlsx
@@ -657,7 +657,7 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>24</v>
@@ -775,7 +775,7 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>37</v>

</xml_diff>